<commit_message>
Add Namibia expedition and frontier balance systems
</commit_message>
<xml_diff>
--- a/resource-rework/resources/RESOURCES.xlsx
+++ b/resource-rework/resources/RESOURCES.xlsx
@@ -206,10 +206,10 @@
         <v>538</v>
       </c>
       <c r="C14">
-        <v>327</v>
+        <v>377</v>
       </c>
       <c r="D14">
-        <v>-211</v>
+        <v>-161</v>
       </c>
     </row>
     <row r="15">
@@ -1430,10 +1430,10 @@
         <v>70</v>
       </c>
       <c r="D77">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E77">
-        <v>-64</v>
+        <v>-52</v>
       </c>
     </row>
     <row r="78">
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10">
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-103</v>
+        <v>-86</v>
       </c>
     </row>
     <row r="12">
@@ -4228,15 +4228,15 @@
         <v>80</v>
       </c>
       <c r="D14">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Counterfactual</t>
+          <t xml:space="preserve">Exception</t>
         </is>
       </c>
       <c r="F14">
-        <v>-49</v>
+        <v>-32</v>
       </c>
     </row>
     <row r="15">
@@ -5170,7 +5170,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-88</v>
+        <v>-67</v>
       </c>
     </row>
     <row r="12">
@@ -5237,15 +5237,15 @@
         <v>70</v>
       </c>
       <c r="D14">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Counterfactual</t>
+          <t xml:space="preserve">Exception</t>
         </is>
       </c>
       <c r="F14">
-        <v>-43</v>
+        <v>-22</v>
       </c>
     </row>
     <row r="15">
@@ -6179,7 +6179,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -6189,7 +6189,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-68</v>
+        <v>-56</v>
       </c>
     </row>
     <row r="12">
@@ -6246,15 +6246,15 @@
         <v>40</v>
       </c>
       <c r="D14">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Exception</t>
         </is>
       </c>
       <c r="F14">
-        <v>-36</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="15">

</xml_diff>